<commit_message>
dates and rounds update
</commit_message>
<xml_diff>
--- a/data/DreamLeague25-26.xlsx
+++ b/data/DreamLeague25-26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kelloggcompany-my.sharepoint.com/personal/bryn_coombe_kellogg_com/Documents/Desktop/Dream League/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="990" documentId="8_{C787F6C9-6D19-48E2-96AB-9D578E0B907B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{071680D5-ED3B-489B-8637-03FDAE99F1D6}"/>
+  <xr:revisionPtr revIDLastSave="1191" documentId="8_{C787F6C9-6D19-48E2-96AB-9D578E0B907B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12189F22-E748-47CA-A971-48C005002AA1}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" state="hidden" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Table!$C$6:$G$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1345" uniqueCount="536">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -1490,9 +1491,6 @@
     <t>RUBEN DIAS</t>
   </si>
   <si>
-    <t>BRSTOL CITY</t>
-  </si>
-  <si>
     <t>MIKEL MERINO</t>
   </si>
   <si>
@@ -1526,9 +1524,6 @@
     <t>NATHANIEL MENDEZ-LAING</t>
   </si>
   <si>
-    <t>MILTON KEYNES</t>
-  </si>
-  <si>
     <t>(6 - 1)</t>
   </si>
   <si>
@@ -1638,6 +1633,21 @@
   </si>
   <si>
     <t>BURTON</t>
+  </si>
+  <si>
+    <t>MATEUS MANE</t>
+  </si>
+  <si>
+    <t>MARCUS BROWNE</t>
+  </si>
+  <si>
+    <t>ARIBIM PEPPLE</t>
+  </si>
+  <si>
+    <t>(3 - 1)</t>
+  </si>
+  <si>
+    <t>Qtr Final Replays</t>
   </si>
 </sst>
 </file>
@@ -3688,11 +3698,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="15">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G5" s="83"/>
       <c r="H5" s="84"/>
-      <c r="I5" s="85"/>
+      <c r="I5" s="85">
+        <v>1</v>
+      </c>
       <c r="J5" s="82"/>
       <c r="K5" s="16" t="str">
         <f>D2</f>
@@ -3704,15 +3716,15 @@
       </c>
       <c r="M5" s="18">
         <f t="shared" ref="M5:M17" si="0">N5-O5</f>
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N5" s="19">
         <f>SUM(F8:F25)</f>
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="O5" s="20">
         <f>SUM(F5:F7)</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="S5" s="102"/>
       <c r="T5" s="101"/>
@@ -3743,11 +3755,11 @@
       </c>
       <c r="N6" s="26">
         <f>SUM(F35:F52)</f>
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="O6" s="27">
         <f>SUM(F32:F34)</f>
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="S6" s="102"/>
       <c r="T6" s="101"/>
@@ -3778,11 +3790,11 @@
       </c>
       <c r="N7" s="26">
         <f>SUM(F62:F79)</f>
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O7" s="27">
         <f>SUM(F59:F61)</f>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S7" s="102"/>
       <c r="T7" s="101"/>
@@ -3818,11 +3830,11 @@
       </c>
       <c r="M8" s="25">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="N8" s="26">
         <f>SUM(F89:F106)</f>
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="O8" s="27">
         <f>SUM(F86:F88)</f>
@@ -3860,15 +3872,15 @@
       </c>
       <c r="M9" s="25">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="N9" s="73">
         <f>SUM(F116:F133)</f>
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="O9" s="74">
         <f>SUM(F113:F115)</f>
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -3877,7 +3889,7 @@
         <v>16</v>
       </c>
       <c r="C10" s="106" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D10" s="106" t="s">
         <v>24</v>
@@ -3906,15 +3918,15 @@
       </c>
       <c r="M10" s="25">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="N10" s="26">
         <f>SUM(F143:F160)</f>
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="O10" s="27">
         <f>SUM(F140:F142)</f>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="R10" s="119"/>
       <c r="S10" s="119"/>
@@ -3955,15 +3967,15 @@
       </c>
       <c r="M11" s="25">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11" s="26">
         <f>SUM(F170:F187)</f>
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O11" s="27">
         <f>SUM(F167:F169)</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S11" s="102"/>
       <c r="T11" s="101"/>
@@ -4004,15 +4016,15 @@
       </c>
       <c r="M12" s="25">
         <f t="shared" si="0"/>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N12" s="73">
         <f>SUM(F197:F214)</f>
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="O12" s="74">
         <f>SUM(F194:F196)</f>
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -4048,15 +4060,15 @@
       </c>
       <c r="M13" s="25">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="N13" s="73">
         <f>SUM(F224:F241)</f>
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="O13" s="74">
         <f>SUM(F221:F223)</f>
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="R13" s="119"/>
       <c r="S13" s="119"/>
@@ -4095,15 +4107,15 @@
       </c>
       <c r="M14" s="25">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N14" s="73">
         <f>SUM(F251:F268)</f>
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="O14" s="74">
         <f>SUM(F248:F250)</f>
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="S14" s="102"/>
       <c r="T14" s="101"/>
@@ -4148,11 +4160,11 @@
       </c>
       <c r="N15" s="26">
         <f>SUM(F278:F295)</f>
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="O15" s="27">
         <f>SUM(F275:F277)</f>
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:22" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -4188,15 +4200,15 @@
       </c>
       <c r="M16" s="25">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N16" s="26">
         <f>SUM(F305:F322)</f>
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O16" s="27">
         <f>SUM(F302:F304)</f>
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:22" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -4230,15 +4242,15 @@
       </c>
       <c r="M17" s="25">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="N17" s="26">
         <f>SUM(F332:F349)</f>
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="O17" s="27">
         <f>SUM(F329:F331)</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R17" s="119"/>
       <c r="S17" s="119"/>
@@ -4281,11 +4293,11 @@
       </c>
       <c r="M18" s="25">
         <f>N18-O18</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="N18" s="26">
         <f>SUM(F359:F376)</f>
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="O18" s="27">
         <f>SUM(F356:F358)</f>
@@ -4341,13 +4353,15 @@
         <v>284</v>
       </c>
       <c r="F20" s="30">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G20" s="87">
         <v>45932</v>
       </c>
       <c r="H20" s="84"/>
-      <c r="I20" s="99"/>
+      <c r="I20" s="99">
+        <v>1</v>
+      </c>
       <c r="J20" s="76"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
@@ -4400,7 +4414,7 @@
         <v>17</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D22" s="28" t="s">
         <v>18</v>
@@ -4496,7 +4510,7 @@
         <v>17</v>
       </c>
       <c r="C25" s="28" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="D25" s="28" t="s">
         <v>74</v>
@@ -4533,7 +4547,7 @@
       </c>
       <c r="F26" s="36">
         <f>SUM(F8:F25)-SUM(F5:F7)</f>
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G26" s="80"/>
       <c r="H26" s="92"/>
@@ -4649,23 +4663,27 @@
       <c r="N31" s="1"/>
       <c r="O31" s="1"/>
     </row>
-    <row r="32" spans="1:22" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" ht="13.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="79"/>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="C32" s="13"/>
-      <c r="D32" s="12" t="s">
+      <c r="C32" s="111"/>
+      <c r="D32" s="110" t="s">
         <v>122</v>
       </c>
-      <c r="E32" s="14">
+      <c r="E32" s="112">
         <v>1</v>
       </c>
-      <c r="F32" s="15">
-        <v>40</v>
-      </c>
-      <c r="G32" s="80"/>
-      <c r="H32" s="94"/>
+      <c r="F32" s="113">
+        <v>44</v>
+      </c>
+      <c r="G32" s="80" t="s">
+        <v>285</v>
+      </c>
+      <c r="H32" s="94">
+        <v>46072</v>
+      </c>
       <c r="I32" s="95"/>
       <c r="J32" s="76"/>
       <c r="K32" s="1"/>
@@ -4676,14 +4694,26 @@
     </row>
     <row r="33" spans="1:22" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="79"/>
-      <c r="B33" s="21"/>
+      <c r="B33" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="86"/>
+      <c r="D33" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E33" s="22" t="s">
+        <v>284</v>
+      </c>
+      <c r="F33" s="21">
+        <v>2</v>
+      </c>
+      <c r="G33" s="86">
+        <v>46072</v>
+      </c>
       <c r="H33" s="94"/>
-      <c r="I33" s="93"/>
+      <c r="I33" s="93">
+        <v>2</v>
+      </c>
       <c r="J33" s="76"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
@@ -4853,7 +4883,7 @@
         <v>1</v>
       </c>
       <c r="F40" s="30">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G40" s="87"/>
       <c r="H40" s="91"/>
@@ -4933,7 +4963,7 @@
         <v>17</v>
       </c>
       <c r="C43" s="28" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="D43" s="28" t="s">
         <v>132</v>
@@ -5082,10 +5112,10 @@
         <v>17</v>
       </c>
       <c r="C48" s="28" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D48" s="28" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="E48" s="29" t="s">
         <v>284</v>
@@ -5173,22 +5203,24 @@
         <v>17</v>
       </c>
       <c r="C51" s="28" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D51" s="28" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="E51" s="29" t="s">
         <v>284</v>
       </c>
       <c r="F51" s="30">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G51" s="91">
         <v>46051</v>
       </c>
       <c r="H51" s="91"/>
-      <c r="I51" s="89"/>
+      <c r="I51" s="89">
+        <v>3</v>
+      </c>
       <c r="J51" s="76"/>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
@@ -5358,11 +5390,13 @@
         <v>4</v>
       </c>
       <c r="F59" s="15">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G59" s="80"/>
       <c r="H59" s="92"/>
-      <c r="I59" s="92"/>
+      <c r="I59" s="92">
+        <v>1</v>
+      </c>
       <c r="J59" s="76"/>
       <c r="K59" s="1"/>
       <c r="L59" s="1"/>
@@ -5712,7 +5746,7 @@
         <v>284</v>
       </c>
       <c r="F73" s="30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G73" s="87">
         <v>45897</v>
@@ -6220,7 +6254,7 @@
         <v>16</v>
       </c>
       <c r="C94" s="106" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="D94" s="106" t="s">
         <v>24</v>
@@ -6251,16 +6285,16 @@
         <v>16</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="D95" s="28" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="E95" s="29" t="s">
         <v>284</v>
       </c>
       <c r="F95" s="30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G95" s="91">
         <v>46065</v>
@@ -6289,11 +6323,13 @@
         <v>19</v>
       </c>
       <c r="F96" s="30">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G96" s="91"/>
       <c r="H96" s="91"/>
-      <c r="I96" s="90"/>
+      <c r="I96" s="90">
+        <v>2</v>
+      </c>
       <c r="J96" s="76"/>
       <c r="K96" s="1"/>
       <c r="L96" s="1"/>
@@ -6382,7 +6418,7 @@
         <v>17</v>
       </c>
       <c r="C100" s="28" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D100" s="28" t="s">
         <v>97</v>
@@ -6457,9 +6493,7 @@
         <v>45918</v>
       </c>
       <c r="H102" s="91"/>
-      <c r="I102" s="90">
-        <v>1</v>
-      </c>
+      <c r="I102" s="90"/>
       <c r="J102" s="76"/>
       <c r="K102" s="1"/>
       <c r="L102" s="1"/>
@@ -6562,7 +6596,7 @@
         <v>17</v>
       </c>
       <c r="C106" s="28" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="D106" s="28" t="s">
         <v>179</v>
@@ -6577,9 +6611,7 @@
         <v>46002</v>
       </c>
       <c r="H106" s="91"/>
-      <c r="I106" s="92">
-        <v>1</v>
-      </c>
+      <c r="I106" s="92"/>
       <c r="J106" s="1"/>
       <c r="K106" s="1"/>
       <c r="L106" s="1"/>
@@ -6598,7 +6630,7 @@
       </c>
       <c r="F107" s="36">
         <f>SUM(F89:F106)-SUM(F86:F88)</f>
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G107" s="80"/>
       <c r="H107" s="92"/>
@@ -6722,11 +6754,13 @@
         <v>1</v>
       </c>
       <c r="F113" s="15">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G113" s="80"/>
       <c r="H113" s="94"/>
-      <c r="I113" s="90"/>
+      <c r="I113" s="90">
+        <v>1</v>
+      </c>
       <c r="J113" s="76"/>
       <c r="K113" s="1"/>
       <c r="L113" s="1"/>
@@ -6783,7 +6817,7 @@
         <v>1</v>
       </c>
       <c r="F116" s="30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G116" s="83"/>
       <c r="H116" s="91"/>
@@ -6939,13 +6973,15 @@
         <v>284</v>
       </c>
       <c r="F122" s="30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G122" s="87">
         <v>45974</v>
       </c>
       <c r="H122" s="91"/>
-      <c r="I122" s="90"/>
+      <c r="I122" s="90">
+        <v>1</v>
+      </c>
       <c r="J122" s="76"/>
       <c r="K122" s="1"/>
       <c r="L122" s="1"/>
@@ -7044,19 +7080,19 @@
     </row>
     <row r="126" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="79"/>
-      <c r="B126" s="28" t="s">
+      <c r="B126" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="C126" s="28" t="s">
+      <c r="C126" s="106" t="s">
         <v>475</v>
       </c>
-      <c r="D126" s="28" t="s">
+      <c r="D126" s="106" t="s">
         <v>206</v>
       </c>
-      <c r="E126" s="29" t="s">
+      <c r="E126" s="107" t="s">
         <v>284</v>
       </c>
-      <c r="F126" s="30">
+      <c r="F126" s="108">
         <v>4</v>
       </c>
       <c r="G126" s="87">
@@ -7079,22 +7115,24 @@
         <v>17</v>
       </c>
       <c r="C127" s="28" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="D127" s="28" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="E127" s="29" t="s">
         <v>284</v>
       </c>
       <c r="F127" s="30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G127" s="87">
         <v>46023</v>
       </c>
       <c r="H127" s="91"/>
-      <c r="I127" s="90"/>
+      <c r="I127" s="90">
+        <v>2</v>
+      </c>
       <c r="J127" s="76"/>
       <c r="K127" s="1"/>
       <c r="L127" s="1"/>
@@ -7179,13 +7217,15 @@
         <v>284</v>
       </c>
       <c r="F130" s="30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G130" s="87">
         <v>46058</v>
       </c>
       <c r="H130" s="91"/>
-      <c r="I130" s="90"/>
+      <c r="I130" s="90">
+        <v>1</v>
+      </c>
       <c r="J130" s="76"/>
       <c r="K130" s="1"/>
       <c r="L130" s="1"/>
@@ -7208,7 +7248,7 @@
         <v>1</v>
       </c>
       <c r="F131" s="30">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G131" s="87"/>
       <c r="H131" s="91"/>
@@ -7266,7 +7306,7 @@
         <v>284</v>
       </c>
       <c r="F133" s="30">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G133" s="87">
         <v>45932</v>
@@ -7291,7 +7331,7 @@
       </c>
       <c r="F134" s="36">
         <f>SUM(F116:F133)-SUM(F113:F115)</f>
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="G134" s="80"/>
       <c r="H134" s="92"/>
@@ -7473,13 +7513,15 @@
         <v>284</v>
       </c>
       <c r="F142" s="21">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G142" s="86">
         <v>45974</v>
       </c>
       <c r="H142" s="92"/>
-      <c r="I142" s="118"/>
+      <c r="I142" s="118">
+        <v>2</v>
+      </c>
       <c r="J142" s="76"/>
       <c r="K142" s="1"/>
       <c r="L142" s="1"/>
@@ -7658,13 +7700,15 @@
         <v>284</v>
       </c>
       <c r="F149" s="30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G149" s="87">
         <v>45974</v>
       </c>
       <c r="H149" s="91"/>
-      <c r="I149" s="90"/>
+      <c r="I149" s="90">
+        <v>1</v>
+      </c>
       <c r="J149" s="76"/>
       <c r="K149" s="1"/>
       <c r="L149" s="1"/>
@@ -7674,13 +7718,27 @@
     </row>
     <row r="150" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="79"/>
-      <c r="B150" s="28"/>
-      <c r="C150" s="28"/>
-      <c r="D150" s="28"/>
-      <c r="E150" s="29"/>
-      <c r="F150" s="30"/>
-      <c r="G150" s="87"/>
-      <c r="H150" s="91"/>
+      <c r="B150" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="C150" s="106" t="s">
+        <v>150</v>
+      </c>
+      <c r="D150" s="106" t="s">
+        <v>68</v>
+      </c>
+      <c r="E150" s="107">
+        <v>1</v>
+      </c>
+      <c r="F150" s="108">
+        <v>5</v>
+      </c>
+      <c r="G150" s="87" t="s">
+        <v>285</v>
+      </c>
+      <c r="H150" s="91">
+        <v>46030</v>
+      </c>
       <c r="I150" s="90"/>
       <c r="J150" s="76"/>
       <c r="K150" s="1"/>
@@ -7691,28 +7749,28 @@
     </row>
     <row r="151" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="79"/>
-      <c r="B151" s="106" t="s">
+      <c r="B151" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C151" s="106" t="s">
-        <v>150</v>
-      </c>
-      <c r="D151" s="106" t="s">
-        <v>68</v>
-      </c>
-      <c r="E151" s="107">
+      <c r="C151" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="D151" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E151" s="29" t="s">
+        <v>284</v>
+      </c>
+      <c r="F151" s="30">
+        <v>4</v>
+      </c>
+      <c r="G151" s="87">
+        <v>46030</v>
+      </c>
+      <c r="H151" s="91"/>
+      <c r="I151" s="90">
         <v>1</v>
       </c>
-      <c r="F151" s="108">
-        <v>5</v>
-      </c>
-      <c r="G151" s="87" t="s">
-        <v>285</v>
-      </c>
-      <c r="H151" s="91">
-        <v>46030</v>
-      </c>
-      <c r="I151" s="90"/>
       <c r="J151" s="76"/>
       <c r="K151" s="1"/>
       <c r="L151" s="1"/>
@@ -7722,25 +7780,27 @@
     </row>
     <row r="152" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="79"/>
-      <c r="B152" s="28" t="s">
+      <c r="B152" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="C152" s="28" t="s">
-        <v>507</v>
-      </c>
-      <c r="D152" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="E152" s="29" t="s">
-        <v>284</v>
-      </c>
-      <c r="F152" s="30">
-        <v>3</v>
-      </c>
-      <c r="G152" s="87">
-        <v>46030</v>
-      </c>
-      <c r="H152" s="91"/>
+      <c r="C152" s="106" t="s">
+        <v>213</v>
+      </c>
+      <c r="D152" s="106" t="s">
+        <v>83</v>
+      </c>
+      <c r="E152" s="107">
+        <v>18</v>
+      </c>
+      <c r="F152" s="108">
+        <v>10</v>
+      </c>
+      <c r="G152" s="83" t="s">
+        <v>285</v>
+      </c>
+      <c r="H152" s="91">
+        <v>46072</v>
+      </c>
       <c r="I152" s="90"/>
       <c r="J152" s="76"/>
       <c r="K152" s="1"/>
@@ -7755,20 +7815,24 @@
         <v>17</v>
       </c>
       <c r="C153" s="28" t="s">
-        <v>213</v>
+        <v>533</v>
       </c>
       <c r="D153" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="E153" s="29">
-        <v>18</v>
+        <v>425</v>
+      </c>
+      <c r="E153" s="29" t="s">
+        <v>284</v>
       </c>
       <c r="F153" s="30">
-        <v>10</v>
-      </c>
-      <c r="G153" s="83"/>
+        <v>2</v>
+      </c>
+      <c r="G153" s="87">
+        <v>46072</v>
+      </c>
       <c r="H153" s="91"/>
-      <c r="I153" s="90"/>
+      <c r="I153" s="90">
+        <v>2</v>
+      </c>
       <c r="J153" s="96"/>
       <c r="K153" s="1"/>
       <c r="L153" s="1"/>
@@ -7844,10 +7908,10 @@
         <v>17</v>
       </c>
       <c r="C156" s="106" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="D156" s="106" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="E156" s="107" t="s">
         <v>284</v>
@@ -7875,10 +7939,10 @@
         <v>17</v>
       </c>
       <c r="C157" s="28" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D157" s="28" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="E157" s="29" t="s">
         <v>284</v>
@@ -7913,11 +7977,13 @@
         <v>25</v>
       </c>
       <c r="F158" s="30">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G158" s="87"/>
       <c r="H158" s="91"/>
-      <c r="I158" s="90"/>
+      <c r="I158" s="90">
+        <v>1</v>
+      </c>
       <c r="J158" s="76"/>
       <c r="K158" s="1"/>
       <c r="L158" s="1"/>
@@ -7962,7 +8028,7 @@
         <v>17</v>
       </c>
       <c r="C160" s="28" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="D160" s="28" t="s">
         <v>20</v>
@@ -7996,7 +8062,7 @@
       </c>
       <c r="F161" s="36">
         <f>SUM(F143:F160)-SUM(F140:F142)</f>
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G161" s="80"/>
       <c r="H161" s="92"/>
@@ -8149,7 +8215,7 @@
         <v>284</v>
       </c>
       <c r="F168" s="21">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G168" s="86">
         <v>46318</v>
@@ -8266,11 +8332,13 @@
         <v>3</v>
       </c>
       <c r="F173" s="30">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G173" s="83"/>
       <c r="H173" s="91"/>
-      <c r="I173" s="90"/>
+      <c r="I173" s="90">
+        <v>1</v>
+      </c>
       <c r="J173" s="76"/>
       <c r="K173" s="1"/>
       <c r="L173" s="1"/>
@@ -8464,7 +8532,7 @@
         <v>17</v>
       </c>
       <c r="C180" s="28" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D180" s="28" t="s">
         <v>20</v>
@@ -8493,7 +8561,7 @@
         <v>17</v>
       </c>
       <c r="C181" s="28" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="D181" s="28" t="s">
         <v>148</v>
@@ -8589,7 +8657,7 @@
         <v>284</v>
       </c>
       <c r="F184" s="30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G184" s="87">
         <v>45953</v>
@@ -8705,7 +8773,7 @@
       </c>
       <c r="F188" s="36">
         <f>SUM(F170:F187)-SUM(F167:F169)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G188" s="87"/>
       <c r="H188" s="91"/>
@@ -8829,7 +8897,7 @@
         <v>1</v>
       </c>
       <c r="F194" s="15">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="G194" s="80"/>
       <c r="H194" s="94"/>
@@ -8961,7 +9029,7 @@
         <v>1</v>
       </c>
       <c r="F200" s="30">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G200" s="83"/>
       <c r="H200" s="90"/>
@@ -9087,13 +9155,13 @@
         <v>272</v>
       </c>
       <c r="D206" s="28" t="s">
-        <v>483</v>
+        <v>87</v>
       </c>
       <c r="E206" s="29">
         <v>1</v>
       </c>
       <c r="F206" s="30">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G206" s="87"/>
       <c r="H206" s="90"/>
@@ -9174,11 +9242,13 @@
         <v>1</v>
       </c>
       <c r="F209" s="30">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G209" s="87"/>
       <c r="H209" s="91"/>
-      <c r="I209" s="90"/>
+      <c r="I209" s="90">
+        <v>2</v>
+      </c>
       <c r="J209" s="76"/>
       <c r="K209" s="1"/>
       <c r="L209" s="1"/>
@@ -9201,7 +9271,7 @@
         <v>1</v>
       </c>
       <c r="F210" s="30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G210" s="87"/>
       <c r="H210" s="90"/>
@@ -9292,7 +9362,7 @@
       </c>
       <c r="F215" s="36">
         <f>SUM(F197:F214)-SUM(F194:F196)</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G215" s="80"/>
       <c r="H215" s="92"/>
@@ -9474,15 +9544,13 @@
         <v>284</v>
       </c>
       <c r="F223" s="21">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G223" s="86">
         <v>46016</v>
       </c>
       <c r="H223" s="92"/>
-      <c r="I223" s="93">
-        <v>3</v>
-      </c>
+      <c r="I223" s="93"/>
       <c r="J223" s="76"/>
       <c r="K223" s="1"/>
       <c r="L223" s="1"/>
@@ -9636,11 +9704,13 @@
         <v>5</v>
       </c>
       <c r="F229" s="30">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G229" s="87"/>
       <c r="H229" s="91"/>
-      <c r="I229" s="89"/>
+      <c r="I229" s="89">
+        <v>1</v>
+      </c>
       <c r="J229" s="76"/>
       <c r="K229" s="1"/>
       <c r="L229" s="1"/>
@@ -9754,7 +9824,7 @@
         <v>36</v>
       </c>
       <c r="F233" s="30">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G233" s="87"/>
       <c r="H233" s="91"/>
@@ -9810,11 +9880,13 @@
         <v>8</v>
       </c>
       <c r="F235" s="30">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G235" s="83"/>
       <c r="H235" s="91"/>
-      <c r="I235" s="89"/>
+      <c r="I235" s="89">
+        <v>1</v>
+      </c>
       <c r="J235" s="76"/>
       <c r="K235" s="1"/>
       <c r="L235" s="1"/>
@@ -9859,7 +9931,7 @@
         <v>17</v>
       </c>
       <c r="C237" s="28" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="D237" s="28" t="s">
         <v>95</v>
@@ -9874,9 +9946,7 @@
         <v>46016</v>
       </c>
       <c r="H237" s="91"/>
-      <c r="I237" s="89">
-        <v>1</v>
-      </c>
+      <c r="I237" s="89"/>
       <c r="J237" s="76"/>
       <c r="K237" s="1"/>
       <c r="L237" s="1"/>
@@ -9930,13 +10000,15 @@
         <v>284</v>
       </c>
       <c r="F239" s="30">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G239" s="87">
         <v>45911</v>
       </c>
       <c r="H239" s="91"/>
-      <c r="I239" s="89"/>
+      <c r="I239" s="89">
+        <v>2</v>
+      </c>
       <c r="J239" s="76"/>
       <c r="K239" s="1"/>
       <c r="L239" s="1"/>
@@ -9989,7 +10061,7 @@
       </c>
       <c r="F242" s="36">
         <f>SUM(F224:F241)-SUM(F221:F223)</f>
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G242" s="80"/>
       <c r="H242" s="92"/>
@@ -10157,13 +10229,13 @@
       </c>
       <c r="C250" s="21"/>
       <c r="D250" s="21" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E250" s="22" t="s">
         <v>284</v>
       </c>
       <c r="F250" s="21">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G250" s="86">
         <v>46037</v>
@@ -10263,7 +10335,7 @@
         <v>1</v>
       </c>
       <c r="F254" s="30">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G254" s="83"/>
       <c r="H254" s="91"/>
@@ -10343,10 +10415,10 @@
         <v>16</v>
       </c>
       <c r="C257" s="28" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D257" s="28" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="E257" s="29" t="s">
         <v>284</v>
@@ -10510,13 +10582,15 @@
         <v>284</v>
       </c>
       <c r="F263" s="30">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G263" s="87">
         <v>45946</v>
       </c>
       <c r="H263" s="91"/>
-      <c r="I263" s="90"/>
+      <c r="I263" s="90">
+        <v>1</v>
+      </c>
       <c r="J263" s="1"/>
       <c r="K263" s="1"/>
       <c r="L263" s="1"/>
@@ -10652,10 +10726,10 @@
         <v>17</v>
       </c>
       <c r="C268" s="28" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="D268" s="28" t="s">
-        <v>495</v>
+        <v>80</v>
       </c>
       <c r="E268" s="29" t="s">
         <v>284</v>
@@ -10686,7 +10760,7 @@
       </c>
       <c r="F269" s="36">
         <f>SUM(F251:F268)-SUM(F248:F250)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G269" s="80"/>
       <c r="H269" s="92"/>
@@ -10839,13 +10913,15 @@
         <v>284</v>
       </c>
       <c r="F276" s="21">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G276" s="86">
         <v>45974</v>
       </c>
       <c r="H276" s="92"/>
-      <c r="I276" s="92"/>
+      <c r="I276" s="92">
+        <v>3</v>
+      </c>
       <c r="J276" s="1"/>
       <c r="K276" s="1"/>
       <c r="L276" s="1"/>
@@ -11131,11 +11207,13 @@
         <v>1</v>
       </c>
       <c r="F288" s="30">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G288" s="87"/>
       <c r="H288" s="91"/>
-      <c r="I288" s="90"/>
+      <c r="I288" s="90">
+        <v>1</v>
+      </c>
       <c r="J288" s="1"/>
       <c r="K288" s="1"/>
       <c r="L288" s="1"/>
@@ -11189,7 +11267,7 @@
         <v>284</v>
       </c>
       <c r="F290" s="30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G290" s="87">
         <v>45946</v>
@@ -11245,11 +11323,13 @@
         <v>1</v>
       </c>
       <c r="F292" s="30">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G292" s="87"/>
       <c r="H292" s="91"/>
-      <c r="I292" s="90"/>
+      <c r="I292" s="90">
+        <v>1</v>
+      </c>
       <c r="J292" s="1"/>
       <c r="K292" s="1"/>
       <c r="L292" s="1"/>
@@ -11501,7 +11581,7 @@
         <v>284</v>
       </c>
       <c r="F304" s="21">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G304" s="87">
         <v>45953</v>
@@ -11524,7 +11604,7 @@
         <v>234</v>
       </c>
       <c r="D305" s="28" t="s">
-        <v>179</v>
+        <v>30</v>
       </c>
       <c r="E305" s="29">
         <v>2</v>
@@ -11623,7 +11703,7 @@
         <v>16</v>
       </c>
       <c r="C309" s="28" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D309" s="28" t="s">
         <v>64</v>
@@ -11743,7 +11823,7 @@
         <v>16</v>
       </c>
       <c r="C313" s="28" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="D313" s="28" t="s">
         <v>86</v>
@@ -11839,13 +11919,15 @@
         <v>284</v>
       </c>
       <c r="F316" s="30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G316" s="87">
         <v>45939</v>
       </c>
       <c r="H316" s="91"/>
-      <c r="I316" s="90"/>
+      <c r="I316" s="90">
+        <v>1</v>
+      </c>
       <c r="J316" s="1"/>
       <c r="K316" s="1"/>
       <c r="L316" s="1"/>
@@ -11948,7 +12030,7 @@
         <v>17</v>
       </c>
       <c r="C320" s="28" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="D320" s="28" t="s">
         <v>80</v>
@@ -12042,7 +12124,7 @@
       </c>
       <c r="F323" s="36">
         <f>SUM(F305:F322)-SUM(F302:F304)</f>
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G323" s="80"/>
       <c r="H323" s="92"/>
@@ -12166,11 +12248,13 @@
         <v>1</v>
       </c>
       <c r="F329" s="15">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G329" s="83"/>
       <c r="H329" s="87"/>
-      <c r="I329" s="90"/>
+      <c r="I329" s="90">
+        <v>1</v>
+      </c>
       <c r="J329" s="1"/>
       <c r="K329" s="1"/>
       <c r="L329" s="1"/>
@@ -12320,7 +12404,7 @@
         <v>16</v>
       </c>
       <c r="C336" s="28" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="D336" s="28" t="s">
         <v>19</v>
@@ -12345,23 +12429,27 @@
     </row>
     <row r="337" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A337" s="79"/>
-      <c r="B337" s="28" t="s">
+      <c r="B337" s="106" t="s">
         <v>16</v>
       </c>
-      <c r="C337" s="28" t="s">
+      <c r="C337" s="106" t="s">
         <v>180</v>
       </c>
-      <c r="D337" s="28" t="s">
+      <c r="D337" s="106" t="s">
         <v>160</v>
       </c>
-      <c r="E337" s="29">
+      <c r="E337" s="107">
         <v>1</v>
       </c>
-      <c r="F337" s="30">
+      <c r="F337" s="108">
         <v>2</v>
       </c>
-      <c r="G337" s="87"/>
-      <c r="H337" s="90"/>
+      <c r="G337" s="87" t="s">
+        <v>285</v>
+      </c>
+      <c r="H337" s="91">
+        <v>46072</v>
+      </c>
       <c r="I337" s="90"/>
       <c r="J337" s="1"/>
       <c r="K337" s="1"/>
@@ -12376,18 +12464,20 @@
         <v>16</v>
       </c>
       <c r="C338" s="28" t="s">
-        <v>279</v>
+        <v>531</v>
       </c>
       <c r="D338" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="E338" s="29">
-        <v>1</v>
+        <v>103</v>
+      </c>
+      <c r="E338" s="29" t="s">
+        <v>284</v>
       </c>
       <c r="F338" s="30">
-        <v>3</v>
-      </c>
-      <c r="G338" s="83"/>
+        <v>0</v>
+      </c>
+      <c r="G338" s="87">
+        <v>46072</v>
+      </c>
       <c r="H338" s="91"/>
       <c r="I338" s="90"/>
       <c r="J338" s="1"/>
@@ -12399,11 +12489,21 @@
     </row>
     <row r="339" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A339" s="79"/>
-      <c r="B339" s="28"/>
-      <c r="C339" s="28"/>
-      <c r="D339" s="28"/>
-      <c r="E339" s="29"/>
-      <c r="F339" s="30"/>
+      <c r="B339" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C339" s="28" t="s">
+        <v>279</v>
+      </c>
+      <c r="D339" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="E339" s="29">
+        <v>1</v>
+      </c>
+      <c r="F339" s="30">
+        <v>3</v>
+      </c>
       <c r="G339" s="87"/>
       <c r="H339" s="91"/>
       <c r="I339" s="90"/>
@@ -12427,23 +12527,27 @@
     </row>
     <row r="341" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A341" s="79"/>
-      <c r="B341" s="28" t="s">
+      <c r="B341" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="C341" s="28" t="s">
+      <c r="C341" s="106" t="s">
         <v>242</v>
       </c>
-      <c r="D341" s="28" t="s">
+      <c r="D341" s="106" t="s">
         <v>206</v>
       </c>
-      <c r="E341" s="29">
+      <c r="E341" s="107">
         <v>1</v>
       </c>
-      <c r="F341" s="30">
+      <c r="F341" s="108">
         <v>1</v>
       </c>
-      <c r="G341" s="83"/>
-      <c r="H341" s="91"/>
+      <c r="G341" s="83" t="s">
+        <v>285</v>
+      </c>
+      <c r="H341" s="91">
+        <v>46072</v>
+      </c>
       <c r="I341" s="90"/>
       <c r="J341" s="1"/>
       <c r="N341" s="1"/>
@@ -12455,20 +12559,24 @@
         <v>17</v>
       </c>
       <c r="C342" s="28" t="s">
-        <v>142</v>
+        <v>532</v>
       </c>
       <c r="D342" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="E342" s="29">
+        <v>156</v>
+      </c>
+      <c r="E342" s="29" t="s">
+        <v>284</v>
+      </c>
+      <c r="F342" s="30">
         <v>1</v>
       </c>
-      <c r="F342" s="30">
-        <v>9</v>
-      </c>
-      <c r="G342" s="87"/>
+      <c r="G342" s="87">
+        <v>46072</v>
+      </c>
       <c r="H342" s="91"/>
-      <c r="I342" s="90"/>
+      <c r="I342" s="90">
+        <v>1</v>
+      </c>
       <c r="J342" s="1"/>
       <c r="N342" s="1"/>
       <c r="O342" s="1"/>
@@ -12479,43 +12587,49 @@
         <v>17</v>
       </c>
       <c r="C343" s="28" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="D343" s="28" t="s">
-        <v>121</v>
+        <v>82</v>
       </c>
       <c r="E343" s="29">
         <v>1</v>
       </c>
       <c r="F343" s="30">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G343" s="87"/>
       <c r="H343" s="91"/>
-      <c r="I343" s="90"/>
+      <c r="I343" s="90">
+        <v>1</v>
+      </c>
       <c r="J343" s="1"/>
       <c r="N343" s="1"/>
       <c r="O343" s="1"/>
     </row>
     <row r="344" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A344" s="79"/>
-      <c r="B344" s="28" t="s">
+      <c r="B344" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="C344" s="28" t="s">
-        <v>280</v>
-      </c>
-      <c r="D344" s="28" t="s">
-        <v>132</v>
-      </c>
-      <c r="E344" s="29">
+      <c r="C344" s="106" t="s">
+        <v>127</v>
+      </c>
+      <c r="D344" s="106" t="s">
+        <v>121</v>
+      </c>
+      <c r="E344" s="107">
         <v>1</v>
       </c>
-      <c r="F344" s="30">
-        <v>10</v>
-      </c>
-      <c r="G344" s="83"/>
-      <c r="H344" s="91"/>
+      <c r="F344" s="108">
+        <v>3</v>
+      </c>
+      <c r="G344" s="87" t="s">
+        <v>285</v>
+      </c>
+      <c r="H344" s="91">
+        <v>46072</v>
+      </c>
       <c r="I344" s="90"/>
       <c r="J344" s="1"/>
       <c r="N344" s="1"/>
@@ -12523,28 +12637,28 @@
     </row>
     <row r="345" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A345" s="79"/>
-      <c r="B345" s="106" t="s">
+      <c r="B345" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C345" s="106" t="s">
-        <v>281</v>
-      </c>
-      <c r="D345" s="106" t="s">
-        <v>84</v>
-      </c>
-      <c r="E345" s="107">
+      <c r="C345" s="28" t="s">
+        <v>430</v>
+      </c>
+      <c r="D345" s="28" t="s">
+        <v>82</v>
+      </c>
+      <c r="E345" s="29" t="s">
+        <v>284</v>
+      </c>
+      <c r="F345" s="30">
         <v>1</v>
       </c>
-      <c r="F345" s="108">
-        <v>0</v>
-      </c>
-      <c r="G345" s="87" t="s">
-        <v>285</v>
-      </c>
-      <c r="H345" s="91">
-        <v>45932</v>
-      </c>
-      <c r="I345" s="90"/>
+      <c r="G345" s="87">
+        <v>46072</v>
+      </c>
+      <c r="H345" s="91"/>
+      <c r="I345" s="90">
+        <v>1</v>
+      </c>
       <c r="J345" s="1"/>
       <c r="N345" s="1"/>
       <c r="O345" s="1"/>
@@ -12555,20 +12669,18 @@
         <v>17</v>
       </c>
       <c r="C346" s="28" t="s">
-        <v>456</v>
+        <v>280</v>
       </c>
       <c r="D346" s="28" t="s">
-        <v>177</v>
-      </c>
-      <c r="E346" s="29" t="s">
-        <v>284</v>
+        <v>132</v>
+      </c>
+      <c r="E346" s="29">
+        <v>1</v>
       </c>
       <c r="F346" s="30">
-        <v>12</v>
-      </c>
-      <c r="G346" s="87">
-        <v>45932</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="G346" s="83"/>
       <c r="H346" s="91"/>
       <c r="I346" s="90"/>
       <c r="J346" s="1"/>
@@ -12577,13 +12689,27 @@
     </row>
     <row r="347" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A347" s="79"/>
-      <c r="B347" s="28"/>
-      <c r="C347" s="28"/>
-      <c r="D347" s="28"/>
-      <c r="E347" s="29"/>
-      <c r="F347" s="30"/>
-      <c r="G347" s="87"/>
-      <c r="H347" s="91"/>
+      <c r="B347" s="106" t="s">
+        <v>17</v>
+      </c>
+      <c r="C347" s="106" t="s">
+        <v>281</v>
+      </c>
+      <c r="D347" s="106" t="s">
+        <v>84</v>
+      </c>
+      <c r="E347" s="107">
+        <v>1</v>
+      </c>
+      <c r="F347" s="108">
+        <v>0</v>
+      </c>
+      <c r="G347" s="87" t="s">
+        <v>285</v>
+      </c>
+      <c r="H347" s="91">
+        <v>45932</v>
+      </c>
       <c r="I347" s="90"/>
       <c r="J347" s="1"/>
       <c r="N347" s="1"/>
@@ -12591,12 +12717,24 @@
     </row>
     <row r="348" spans="1:15" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A348" s="79"/>
-      <c r="B348" s="28"/>
-      <c r="C348" s="28"/>
-      <c r="D348" s="28"/>
-      <c r="E348" s="29"/>
-      <c r="F348" s="30"/>
-      <c r="G348" s="87"/>
+      <c r="B348" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C348" s="28" t="s">
+        <v>456</v>
+      </c>
+      <c r="D348" s="28" t="s">
+        <v>177</v>
+      </c>
+      <c r="E348" s="29" t="s">
+        <v>284</v>
+      </c>
+      <c r="F348" s="30">
+        <v>13</v>
+      </c>
+      <c r="G348" s="87">
+        <v>45932</v>
+      </c>
       <c r="H348" s="91"/>
       <c r="I348" s="90"/>
       <c r="J348" s="1"/>
@@ -12628,7 +12766,7 @@
       </c>
       <c r="F350" s="36">
         <f>SUM(F332:F349)-SUM(F329:F331)</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G350" s="83"/>
       <c r="H350" s="90"/>
@@ -12753,7 +12891,7 @@
         <v>4</v>
       </c>
       <c r="F359" s="30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G359" s="1"/>
       <c r="H359" s="1"/>
@@ -12806,7 +12944,7 @@
         <v>32</v>
       </c>
       <c r="F362" s="30">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G362" s="1"/>
       <c r="H362" s="1"/>
@@ -12843,7 +12981,7 @@
         <v>16</v>
       </c>
       <c r="C364" s="28" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D364" s="28" t="s">
         <v>18</v>
@@ -12976,11 +13114,13 @@
         <v>5</v>
       </c>
       <c r="F370" s="30">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G370" s="103"/>
       <c r="H370" s="1"/>
-      <c r="I370" s="1"/>
+      <c r="I370" s="1">
+        <v>2</v>
+      </c>
       <c r="J370" s="1"/>
     </row>
     <row r="371" spans="2:10" ht="13.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -13013,7 +13153,7 @@
         <v>17</v>
       </c>
       <c r="C372" s="28" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="D372" s="28" t="s">
         <v>288</v>
@@ -13125,7 +13265,7 @@
       </c>
       <c r="F377" s="36">
         <f>SUM(F359:F376)-SUM(F356:F358)</f>
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G377" s="1"/>
       <c r="H377" s="1"/>
@@ -13494,19 +13634,19 @@
         <v>1</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>98</v>
+        <v>51</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>233</v>
+        <v>203</v>
       </c>
       <c r="E7" s="25">
         <v>35</v>
       </c>
       <c r="F7" s="26">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="G7" s="27">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="H7" s="117"/>
       <c r="I7" s="41"/>
@@ -13519,19 +13659,19 @@
         <v>2</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="D8" s="55" t="s">
-        <v>198</v>
+        <v>233</v>
       </c>
       <c r="E8" s="25">
-        <v>31</v>
-      </c>
-      <c r="F8" s="26">
-        <v>64</v>
-      </c>
-      <c r="G8" s="27">
         <v>33</v>
+      </c>
+      <c r="F8" s="56">
+        <v>83</v>
+      </c>
+      <c r="G8" s="57">
+        <v>50</v>
       </c>
       <c r="H8" s="52"/>
       <c r="I8" s="41"/>
@@ -13544,19 +13684,19 @@
         <v>3</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>1</v>
+        <v>32</v>
+      </c>
+      <c r="D9" s="55" t="s">
+        <v>31</v>
       </c>
       <c r="E9" s="25">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F9" s="26">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="G9" s="27">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="H9" s="52"/>
       <c r="I9" s="41"/>
@@ -13569,19 +13709,19 @@
         <v>4</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="55" t="s">
+        <v>198</v>
+      </c>
+      <c r="E10" s="25">
         <v>31</v>
       </c>
-      <c r="E10" s="25">
-        <v>29</v>
-      </c>
       <c r="F10" s="26">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G10" s="27">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="H10" s="117"/>
       <c r="I10" s="41"/>
@@ -13594,19 +13734,19 @@
         <v>5</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="55" t="s">
-        <v>203</v>
+        <v>27</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>15</v>
       </c>
       <c r="E11" s="25">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F11" s="26">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="G11" s="27">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="H11" s="117"/>
       <c r="I11" s="41"/>
@@ -13619,19 +13759,19 @@
         <v>6</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E12" s="25">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F12" s="26">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="G12" s="27">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="H12" s="52"/>
       <c r="I12" s="41"/>
@@ -13646,17 +13786,17 @@
       <c r="C13" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="55" t="s">
+      <c r="D13" s="24" t="s">
         <v>267</v>
       </c>
       <c r="E13" s="25">
-        <v>20</v>
-      </c>
-      <c r="F13" s="56">
-        <v>70</v>
-      </c>
-      <c r="G13" s="57">
-        <v>50</v>
+        <v>23</v>
+      </c>
+      <c r="F13" s="26">
+        <v>77</v>
+      </c>
+      <c r="G13" s="27">
+        <v>54</v>
       </c>
       <c r="H13" s="117"/>
       <c r="I13" s="41"/>
@@ -13671,17 +13811,17 @@
       <c r="C14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="55" t="s">
         <v>188</v>
       </c>
       <c r="E14" s="25">
         <v>20</v>
       </c>
-      <c r="F14" s="26">
-        <v>60</v>
-      </c>
-      <c r="G14" s="27">
-        <v>40</v>
+      <c r="F14" s="56">
+        <v>66</v>
+      </c>
+      <c r="G14" s="57">
+        <v>46</v>
       </c>
       <c r="H14" s="117"/>
       <c r="I14" s="41"/>
@@ -13694,19 +13834,19 @@
         <v>9</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>66</v>
+        <v>244</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E15" s="25">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F15" s="26">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G15" s="27">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H15" s="117"/>
       <c r="I15" s="41"/>
@@ -13719,19 +13859,19 @@
         <v>10</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="D16" s="55" t="s">
-        <v>245</v>
+        <v>66</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>243</v>
       </c>
       <c r="E16" s="25">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F16" s="26">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G16" s="27">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H16" s="52"/>
       <c r="I16" s="41"/>
@@ -13746,17 +13886,17 @@
       <c r="C17" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D17" s="55" t="s">
+      <c r="D17" s="24" t="s">
         <v>140</v>
       </c>
       <c r="E17" s="25">
         <v>8</v>
       </c>
-      <c r="F17" s="56">
-        <v>54</v>
-      </c>
-      <c r="G17" s="57">
-        <v>46</v>
+      <c r="F17" s="26">
+        <v>58</v>
+      </c>
+      <c r="G17" s="27">
+        <v>50</v>
       </c>
       <c r="H17" s="52"/>
       <c r="I17" s="41"/>
@@ -13775,13 +13915,13 @@
         <v>222</v>
       </c>
       <c r="E18" s="25">
-        <v>5</v>
-      </c>
-      <c r="F18" s="56">
-        <v>60</v>
-      </c>
-      <c r="G18" s="57">
-        <v>55</v>
+        <v>4</v>
+      </c>
+      <c r="F18" s="26">
+        <v>62</v>
+      </c>
+      <c r="G18" s="27">
+        <v>58</v>
       </c>
       <c r="H18" s="52"/>
       <c r="I18" s="41"/>
@@ -13796,17 +13936,17 @@
       <c r="C19" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="55" t="s">
         <v>34</v>
       </c>
       <c r="E19" s="25">
-        <v>3</v>
-      </c>
-      <c r="F19" s="26">
-        <v>45</v>
-      </c>
-      <c r="G19" s="27">
-        <v>42</v>
+        <v>4</v>
+      </c>
+      <c r="F19" s="56">
+        <v>47</v>
+      </c>
+      <c r="G19" s="57">
+        <v>43</v>
       </c>
       <c r="H19" s="52"/>
       <c r="I19" s="41"/>
@@ -13825,13 +13965,13 @@
         <v>53</v>
       </c>
       <c r="E20" s="25">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F20" s="26">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G20" s="27">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H20" s="117"/>
       <c r="I20" s="41"/>
@@ -13884,7 +14024,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:IW29"/>
+  <dimension ref="A1:IW31"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="33.296875" style="38" customWidth="1"/>
@@ -13946,10 +14086,10 @@
         <v>467</v>
       </c>
       <c r="I4" s="38" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="J4" s="38" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -13963,7 +14103,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="64" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="E5" s="68" t="s">
         <v>267</v>
@@ -13972,13 +14112,13 @@
         <v>3</v>
       </c>
       <c r="G5" s="64" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="I5" s="38" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14001,13 +14141,13 @@
         <v>3</v>
       </c>
       <c r="G6" s="64" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="I6" s="38" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14030,13 +14170,13 @@
         <v>-1</v>
       </c>
       <c r="G7" s="100" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="I7" s="38" t="s">
         <v>40</v>
       </c>
       <c r="J7" s="38" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14085,7 +14225,7 @@
         <v>467</v>
       </c>
       <c r="I9" s="38" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -14103,7 +14243,7 @@
     <row r="11" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="67"/>
       <c r="B11" s="63" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C11" s="68"/>
       <c r="D11" s="64"/>
@@ -14164,13 +14304,21 @@
       <c r="B15" s="65" t="s">
         <v>233</v>
       </c>
-      <c r="C15" s="68"/>
-      <c r="D15" s="64"/>
+      <c r="C15" s="68">
+        <v>1</v>
+      </c>
+      <c r="D15" s="64" t="s">
+        <v>433</v>
+      </c>
       <c r="E15" s="65" t="s">
         <v>222</v>
       </c>
-      <c r="F15" s="68"/>
-      <c r="G15" s="64"/>
+      <c r="F15" s="68">
+        <v>1</v>
+      </c>
+      <c r="G15" s="64" t="s">
+        <v>433</v>
+      </c>
     </row>
     <row r="16" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="67" t="s">
@@ -14179,28 +14327,44 @@
       <c r="B16" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="68"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="65" t="s">
-        <v>530</v>
-      </c>
-      <c r="F16" s="68"/>
-      <c r="G16" s="64"/>
+      <c r="C16" s="68">
+        <v>2</v>
+      </c>
+      <c r="D16" s="64" t="s">
+        <v>431</v>
+      </c>
+      <c r="E16" s="70" t="s">
+        <v>528</v>
+      </c>
+      <c r="F16" s="69">
+        <v>1</v>
+      </c>
+      <c r="G16" s="100" t="s">
+        <v>438</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="67" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="65" t="s">
+      <c r="B17" s="70" t="s">
         <v>243</v>
       </c>
-      <c r="C17" s="68"/>
-      <c r="D17" s="64"/>
+      <c r="C17" s="69">
+        <v>2</v>
+      </c>
+      <c r="D17" s="100" t="s">
+        <v>534</v>
+      </c>
       <c r="E17" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="68"/>
-      <c r="G17" s="64"/>
+      <c r="F17" s="68">
+        <v>3</v>
+      </c>
+      <c r="G17" s="64" t="s">
+        <v>522</v>
+      </c>
     </row>
     <row r="18" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="67" t="s">
@@ -14209,13 +14373,21 @@
       <c r="B18" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C18" s="68"/>
-      <c r="D18" s="64"/>
-      <c r="E18" s="65" t="s">
+      <c r="C18" s="68">
+        <v>0</v>
+      </c>
+      <c r="D18" s="64" t="s">
+        <v>436</v>
+      </c>
+      <c r="E18" s="70" t="s">
         <v>198</v>
       </c>
-      <c r="F18" s="68"/>
-      <c r="G18" s="64"/>
+      <c r="F18" s="69">
+        <v>-1</v>
+      </c>
+      <c r="G18" s="100" t="s">
+        <v>437</v>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="63"/>
@@ -14225,101 +14397,127 @@
       <c r="F19" s="66"/>
       <c r="G19" s="40"/>
     </row>
-    <row r="20" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="65"/>
-      <c r="C20" s="64"/>
-      <c r="D20" s="61"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="66"/>
-      <c r="G20" s="40"/>
-    </row>
-    <row r="21" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="63" t="s">
+    <row r="20" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="67"/>
+      <c r="B20" s="63" t="s">
+        <v>535</v>
+      </c>
+      <c r="C20" s="68"/>
+      <c r="D20" s="64"/>
+      <c r="E20" s="65"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="64"/>
+    </row>
+    <row r="21" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="67" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="68" t="s">
+        <v>222</v>
+      </c>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
+      <c r="E21" s="68" t="s">
+        <v>233</v>
+      </c>
+      <c r="F21" s="64"/>
+      <c r="G21" s="64"/>
+    </row>
+    <row r="22" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="65"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="61"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="66"/>
+      <c r="G22" s="40"/>
+    </row>
+    <row r="23" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="63" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="66"/>
-      <c r="D21" s="61"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="66"/>
-      <c r="G21" s="40"/>
-    </row>
-    <row r="22" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="67" t="s">
+      <c r="C23" s="66"/>
+      <c r="D23" s="61"/>
+      <c r="E23" s="40"/>
+      <c r="F23" s="66"/>
+      <c r="G23" s="40"/>
+    </row>
+    <row r="24" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="67" t="s">
         <v>77</v>
       </c>
-      <c r="B22" s="70"/>
-      <c r="C22" s="69"/>
-      <c r="D22" s="100"/>
-      <c r="E22" s="65"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="64"/>
-    </row>
-    <row r="23" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="67" t="s">
+      <c r="B24" s="70"/>
+      <c r="C24" s="69"/>
+      <c r="D24" s="100"/>
+      <c r="E24" s="65"/>
+      <c r="F24" s="68"/>
+      <c r="G24" s="64"/>
+    </row>
+    <row r="25" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="67" t="s">
         <v>78</v>
       </c>
-      <c r="B23" s="65"/>
-      <c r="C23" s="68"/>
-      <c r="D23" s="64"/>
-      <c r="E23" s="70"/>
-      <c r="F23" s="69"/>
-      <c r="G23" s="100"/>
-    </row>
-    <row r="24" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="65"/>
-      <c r="C24" s="65"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-    </row>
-    <row r="25" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="65"/>
+      <c r="C25" s="68"/>
+      <c r="D25" s="64"/>
+      <c r="E25" s="70"/>
+      <c r="F25" s="69"/>
+      <c r="G25" s="100"/>
+    </row>
+    <row r="26" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="65"/>
+      <c r="C26" s="65"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+    </row>
+    <row r="27" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="65"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-    </row>
-    <row r="26" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="67" t="s">
-        <v>110</v>
-      </c>
-      <c r="B26" s="65"/>
-      <c r="C26" s="68"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="70"/>
-      <c r="F26" s="69"/>
-      <c r="G26" s="100"/>
-    </row>
-    <row r="27" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="40"/>
-      <c r="C27" s="40"/>
+      <c r="C27" s="65"/>
       <c r="D27" s="64"/>
-      <c r="E27" s="40"/>
+      <c r="E27" s="65"/>
       <c r="F27" s="40"/>
       <c r="G27" s="40"/>
     </row>
-    <row r="28" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="63" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="K28" s="98"/>
-    </row>
-    <row r="29" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="65"/>
+    <row r="28" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="67" t="s">
+        <v>110</v>
+      </c>
+      <c r="B28" s="65"/>
+      <c r="C28" s="68"/>
+      <c r="D28" s="64"/>
+      <c r="E28" s="70"/>
+      <c r="F28" s="69"/>
+      <c r="G28" s="100"/>
+    </row>
+    <row r="29" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="40"/>
       <c r="C29" s="40"/>
-      <c r="D29" s="40"/>
+      <c r="D29" s="64"/>
       <c r="E29" s="40"/>
       <c r="F29" s="40"/>
       <c r="G29" s="40"/>
+    </row>
+    <row r="30" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="63" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" s="40"/>
+      <c r="D30" s="40"/>
+      <c r="E30" s="40"/>
+      <c r="F30" s="40"/>
+      <c r="G30" s="40"/>
+      <c r="K30" s="98"/>
+    </row>
+    <row r="31" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="65"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="40"/>
+      <c r="E31" s="40"/>
+      <c r="F31" s="40"/>
+      <c r="G31" s="40"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15621,7 +15819,7 @@
         <v>0</v>
       </c>
       <c r="D36" s="100" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E36" s="65" t="s">
         <v>233</v>
@@ -15630,7 +15828,7 @@
         <v>4</v>
       </c>
       <c r="G36" s="64" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="H36" s="38"/>
       <c r="I36" s="38"/>
@@ -15713,7 +15911,7 @@
         <v>5</v>
       </c>
       <c r="D39" s="64" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="E39" s="70" t="s">
         <v>233</v>
@@ -16438,7 +16636,7 @@
       </c>
       <c r="K6">
         <f>COUNTIF(Stats!D:D,'Player Count'!J6)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="109"/>
       <c r="N6" s="67" t="s">
@@ -16495,7 +16693,7 @@
       </c>
       <c r="G8">
         <f>COUNTIF(Stats!D:D,'Player Count'!F8)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" t="s">
         <v>345</v>
@@ -16534,7 +16732,7 @@
       </c>
       <c r="K9">
         <f>COUNTIF(Stats!D:D,'Player Count'!J9)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M9" s="109"/>
       <c r="N9" t="s">
@@ -16926,7 +17124,7 @@
       </c>
       <c r="O21">
         <f>COUNTIF(Stats!D:D,'Player Count'!N21)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q21" s="109"/>
     </row>
@@ -16950,7 +17148,7 @@
       </c>
       <c r="K22">
         <f>COUNTIF(Stats!D:D,'Player Count'!J22)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M22" s="109"/>
       <c r="N22" s="67" t="s">
@@ -17032,7 +17230,7 @@
       </c>
       <c r="C25">
         <f>COUNTIF(Stats!D:D,'Player Count'!B25)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" t="s">
         <v>338</v>
@@ -17064,7 +17262,7 @@
       </c>
       <c r="C26" s="78">
         <f>SUM(C6:C25)</f>
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F26" t="s">
         <v>339</v>
@@ -17146,21 +17344,21 @@
       </c>
       <c r="G29">
         <f>COUNTIF(Stats!D:D,'Player Count'!F29)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J29" s="67" t="s">
         <v>367</v>
       </c>
       <c r="K29">
         <f>COUNTIF(Stats!D:D,'Player Count'!J29)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N29" t="s">
         <v>390</v>
       </c>
       <c r="O29">
         <f>COUNTIF(Stats!D:D,'Player Count'!N29)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.3">
@@ -17169,14 +17367,14 @@
       </c>
       <c r="G30" s="78">
         <f>SUM(G6:G29)</f>
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="J30" s="78" t="s">
         <v>317</v>
       </c>
       <c r="K30" s="78">
         <f>SUM(K6:K29)</f>
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N30" s="78" t="s">
         <v>317</v>
@@ -17192,28 +17390,28 @@
       </c>
       <c r="C38" s="114">
         <f>C26/SUM(C26,G30,K30,O30)</f>
-        <v>0.37444933920704848</v>
+        <v>0.36752136752136755</v>
       </c>
       <c r="D38" s="114"/>
       <c r="E38" s="114"/>
       <c r="F38" s="114"/>
       <c r="G38" s="114">
         <f>G30/SUM(C26,G30,K30,O30)</f>
-        <v>0.27312775330396477</v>
+        <v>0.27350427350427353</v>
       </c>
       <c r="H38" s="114"/>
       <c r="I38" s="114"/>
       <c r="J38" s="114"/>
       <c r="K38" s="114">
         <f>K30/SUM(C26,G30,K30,O30)</f>
-        <v>0.1894273127753304</v>
+        <v>0.20085470085470086</v>
       </c>
       <c r="L38" s="114"/>
       <c r="M38" s="114"/>
       <c r="N38" s="114"/>
       <c r="O38" s="114">
         <f>O30/SUM(C26,G30,K30,O30)</f>
-        <v>0.16299559471365638</v>
+        <v>0.15811965811965811</v>
       </c>
     </row>
   </sheetData>

</xml_diff>